<commit_message>
PatchTST experiments Decomp MoE AND Patch MoE
</commit_message>
<xml_diff>
--- a/trend_methods_comparisons.xlsx
+++ b/trend_methods_comparisons.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\TS_Research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8AD3911-6A66-45AA-815E-DC37894D47D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2353158-D226-438B-9CB7-9875574E2E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20835" yWindow="3585" windowWidth="19095" windowHeight="13350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3000" yWindow="3750" windowWidth="19095" windowHeight="13350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="univariate" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -131,11 +131,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -444,18 +444,18 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2" t="s">
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
@@ -495,368 +495,368 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>6.0653101652860641E-2</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>5.9135306626558297E-2</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <v>6.0881868004798889E-2</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <v>6.0331270098686218E-2</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <v>0.18992419540882111</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="2">
         <v>0.18780592083930969</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="2">
         <v>0.19066256284713751</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="2">
         <v>0.18958905339241031</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
+      <c r="A5" s="3"/>
       <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>7.4847981333732605E-2</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>7.3867104947566986E-2</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>7.4000835418701172E-2</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="2">
         <v>7.4429236352443695E-2</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="2">
         <v>0.2138644605875015</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="2">
         <v>0.21283166110515589</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="2">
         <v>0.2129734605550766</v>
       </c>
-      <c r="J5" s="3">
+      <c r="J5" s="2">
         <v>0.21349926292896271</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
+      <c r="A6" s="3"/>
       <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>8.2939170300960541E-2</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>8.2783102989196777E-2</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <v>8.3175025880336761E-2</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="2">
         <v>8.2250989973545074E-2</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="2">
         <v>0.22957128286361689</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="2">
         <v>0.2295078635215759</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="2">
         <v>0.23002217710018161</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="2">
         <v>0.22852399945259089</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
+      <c r="A7" s="3"/>
       <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>9.210088849067688E-2</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>8.7211035192012787E-2</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <v>8.7761126458644867E-2</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="2">
         <v>8.6717031896114349E-2</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="2">
         <v>0.23955006897449491</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="2">
         <v>0.234220951795578</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="2">
         <v>0.23482601344585419</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7" s="2">
         <v>0.23346953094005579</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>0.27822154760360718</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>0.2468362748622894</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <v>0.2323103845119476</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <v>0.23970293998718259</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="2">
         <v>0.3761809766292572</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="2">
         <v>0.35133877396583563</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="2">
         <v>0.33737865090370178</v>
       </c>
-      <c r="J8" s="3">
+      <c r="J8" s="2">
         <v>0.34523141384124761</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
+      <c r="A9" s="3"/>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <v>0.32062241435050959</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>0.31422403454780579</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="2">
         <v>0.28217679262161249</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="2">
         <v>0.28519684076309199</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="2">
         <v>0.40664035081863398</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="2">
         <v>0.39829480648040771</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="2">
         <v>0.37513938546180731</v>
       </c>
-      <c r="J9" s="3">
+      <c r="J9" s="2">
         <v>0.37566617131233221</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
+      <c r="A10" s="3"/>
       <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <v>0.35428828001022339</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>0.33493760228157038</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="2">
         <v>0.31303119659423828</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <v>0.32257622480392462</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="2">
         <v>0.42650720477104193</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="2">
         <v>0.40424624085426331</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="2">
         <v>0.39411410689353937</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J10" s="2">
         <v>0.39806616306304932</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
+      <c r="A11" s="3"/>
       <c r="B11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>0.39630973339080811</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>0.39119666814804083</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="2">
         <v>0.36075320839881903</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="2">
         <v>0.35400506854057312</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="2">
         <v>0.46566715836524958</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="2">
         <v>0.45727863907814031</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="2">
         <v>0.44121983647346502</v>
       </c>
-      <c r="J11" s="3">
+      <c r="J11" s="2">
         <v>0.43900910019874573</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="2">
         <v>0.29187795519828802</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <v>0.2014200687408447</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="2">
         <v>0.18434713780879969</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="2">
         <v>0.17740802466869349</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="2">
         <v>0.40832436084747309</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="2">
         <v>0.30799403786659241</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="2">
         <v>0.28715837001800543</v>
       </c>
-      <c r="J12" s="3">
+      <c r="J12" s="2">
         <v>0.2810981273651123</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
+      <c r="A13" s="3"/>
       <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="2">
         <v>0.29856470227241522</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="2">
         <v>0.20748123526573181</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="2">
         <v>0.19281201064586639</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="2">
         <v>0.18706659972667691</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="2">
         <v>0.41289883852004999</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="2">
         <v>0.31261855363845831</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="2">
         <v>0.29487830400466919</v>
       </c>
-      <c r="J13" s="3">
+      <c r="J13" s="2">
         <v>0.29218336939811712</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
+      <c r="A14" s="3"/>
       <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="2">
         <v>0.30329647660255432</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="2">
         <v>0.21069060266017911</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="2">
         <v>0.1994637995958328</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="2">
         <v>0.19072908163070679</v>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" s="2">
         <v>0.41686034202575678</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="2">
         <v>0.31909322738647461</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="2">
         <v>0.30647677183151251</v>
       </c>
-      <c r="J14" s="3">
+      <c r="J14" s="2">
         <v>0.29779267311096191</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
+      <c r="A15" s="3"/>
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="2">
         <v>0.30946424603462219</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <v>0.22766339778900149</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="2">
         <v>0.2060439735651016</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="2">
         <v>0.20375575125217441</v>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="2">
         <v>0.42015472054481512</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="2">
         <v>0.3391132652759552</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="2">
         <v>0.31493577361106873</v>
       </c>
-      <c r="J15" s="3">
+      <c r="J15" s="2">
         <v>0.31192770600318909</v>
       </c>
     </row>

</xml_diff>